<commit_message>
data(DE): rebuild 2018 power production and demand from statistics; add Z_Import_Biomass, import eligibility per Land, Berlin gas link
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file_DE.xlsx
+++ b/Conversion Script/Set_filter_file_DE.xlsx
@@ -1020,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B154"/>
+  <dimension ref="A1:B155"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2565,6 +2565,16 @@
         </is>
       </c>
       <c r="B154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Z_Import_Biomass</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
data: district-heat gas boiler HD_Gas_Boiler
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Conversion Script/Set_filter_file_DE.xlsx
+++ b/Conversion Script/Set_filter_file_DE.xlsx
@@ -1020,7 +1020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B155"/>
+  <dimension ref="A1:B156"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="30" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -2575,6 +2575,16 @@
         </is>
       </c>
       <c r="B155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>HD_Gas_Boiler</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>